<commit_message>
Okno serwisowe - aktualizacja plików Excel
</commit_message>
<xml_diff>
--- a/assets/excel/en/global_sdg_indicators.xlsx
+++ b/assets/excel/en/global_sdg_indicators.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sidwab\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\niewiadomskaew\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729ECAD9-EDFC-4040-88AA-FFE102150A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB68C29B-5104-4287-8E16-368DB0C5ADC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SDGs_1-17" sheetId="1" r:id="rId1"/>
@@ -1729,7 +1729,7 @@
     <t>100% deaths registration</t>
   </si>
   <si>
-    <t>Last update: 10-02-2026, 09:34</t>
+    <t>Last update: 24-02-2026, 08:36</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Okno serwisowe 10.03 - aktualizacja excel
</commit_message>
<xml_diff>
--- a/assets/excel/en/global_sdg_indicators.xlsx
+++ b/assets/excel/en/global_sdg_indicators.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\niewiadomskaew\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dregerj\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB68C29B-5104-4287-8E16-368DB0C5ADC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD0C22C0-2E09-4E0C-AB67-95CFA5FF22C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SDGs_1-17" sheetId="1" r:id="rId1"/>
@@ -1729,7 +1729,7 @@
     <t>100% deaths registration</t>
   </si>
   <si>
-    <t>Last update: 24-02-2026, 08:36</t>
+    <t>Last update: 10-03-2026, 12:34</t>
   </si>
 </sst>
 </file>
@@ -6304,49 +6304,51 @@
       <c r="E68" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F68" s="4">
+      <c r="F68" s="5">
         <v>451.8</v>
       </c>
-      <c r="G68" s="4">
+      <c r="G68" s="5">
         <v>440.9</v>
       </c>
-      <c r="H68" s="4">
+      <c r="H68" s="5">
         <v>460.8</v>
       </c>
-      <c r="I68" s="4">
+      <c r="I68" s="5">
         <v>460.8</v>
       </c>
-      <c r="J68" s="4">
+      <c r="J68" s="5">
         <v>441.1</v>
       </c>
-      <c r="K68" s="4">
+      <c r="K68" s="5">
         <v>469</v>
       </c>
-      <c r="L68" s="4">
+      <c r="L68" s="5">
         <v>437.1</v>
       </c>
-      <c r="M68" s="4">
+      <c r="M68" s="5">
         <v>434.8</v>
       </c>
-      <c r="N68" s="4">
+      <c r="N68" s="5">
         <v>437.2</v>
       </c>
-      <c r="O68" s="4">
+      <c r="O68" s="5">
         <v>421</v>
       </c>
-      <c r="P68" s="4">
+      <c r="P68" s="5">
         <v>457.2</v>
       </c>
-      <c r="Q68" s="4">
+      <c r="Q68" s="5">
         <v>475.8</v>
       </c>
-      <c r="R68" s="4">
+      <c r="R68" s="5">
         <v>426.2</v>
       </c>
-      <c r="S68" s="4">
+      <c r="S68" s="5">
         <v>400.4</v>
       </c>
-      <c r="T68" s="3"/>
+      <c r="T68" s="5">
+        <v>400.02</v>
+      </c>
       <c r="U68" s="2" t="s">
         <v>27</v>
       </c>
@@ -6409,7 +6411,9 @@
       <c r="S69" s="4">
         <v>25.7</v>
       </c>
-      <c r="T69" s="3"/>
+      <c r="T69" s="4">
+        <v>24.3</v>
+      </c>
       <c r="U69" s="2" t="s">
         <v>27</v>
       </c>
@@ -6472,7 +6476,9 @@
       <c r="S70" s="4">
         <v>264.39999999999998</v>
       </c>
-      <c r="T70" s="3"/>
+      <c r="T70" s="4">
+        <v>265.39999999999998</v>
+      </c>
       <c r="U70" s="2" t="s">
         <v>27</v>
       </c>
@@ -6527,15 +6533,17 @@
         <v>22.9</v>
       </c>
       <c r="Q71" s="4">
-        <v>25.4</v>
+        <v>25.5</v>
       </c>
       <c r="R71" s="4">
-        <v>24.6</v>
+        <v>26.6</v>
       </c>
       <c r="S71" s="4">
-        <v>25.7</v>
-      </c>
-      <c r="T71" s="3"/>
+        <v>25.8</v>
+      </c>
+      <c r="T71" s="4">
+        <v>25.3</v>
+      </c>
       <c r="U71" s="2" t="s">
         <v>27</v>
       </c>
@@ -6598,7 +6606,9 @@
       <c r="S72" s="4">
         <v>12.1</v>
       </c>
-      <c r="T72" s="3"/>
+      <c r="T72" s="4">
+        <v>11.6</v>
+      </c>
       <c r="U72" s="2" t="s">
         <v>27</v>
       </c>
@@ -6661,7 +6671,9 @@
       <c r="S73" s="4">
         <v>21.4</v>
       </c>
-      <c r="T73" s="3"/>
+      <c r="T73" s="4">
+        <v>20.7</v>
+      </c>
       <c r="U73" s="2" t="s">
         <v>27</v>
       </c>
@@ -6724,7 +6736,9 @@
       <c r="S74" s="4">
         <v>3.4</v>
       </c>
-      <c r="T74" s="3"/>
+      <c r="T74" s="4">
+        <v>3.1</v>
+      </c>
       <c r="U74" s="2" t="s">
         <v>27</v>
       </c>
@@ -6852,7 +6866,9 @@
       <c r="S76" s="4">
         <v>5</v>
       </c>
-      <c r="T76" s="3"/>
+      <c r="T76" s="4">
+        <v>5.0999999999999996</v>
+      </c>
       <c r="U76" s="2" t="s">
         <v>119</v>
       </c>
@@ -7722,9 +7738,11 @@
         <v>34.799999999999997</v>
       </c>
       <c r="S92" s="4">
-        <v>37.6</v>
-      </c>
-      <c r="T92" s="3"/>
+        <v>36.5</v>
+      </c>
+      <c r="T92" s="4">
+        <v>37.700000000000003</v>
+      </c>
       <c r="U92" s="2" t="s">
         <v>27</v>
       </c>
@@ -7767,9 +7785,11 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="S93" s="4">
-        <v>9.8000000000000007</v>
-      </c>
-      <c r="T93" s="3"/>
+        <v>9.6</v>
+      </c>
+      <c r="T93" s="4">
+        <v>9.9</v>
+      </c>
       <c r="U93" s="2" t="s">
         <v>27</v>
       </c>
@@ -7814,7 +7834,9 @@
       <c r="S94" s="4">
         <v>65</v>
       </c>
-      <c r="T94" s="3"/>
+      <c r="T94" s="4">
+        <v>66.3</v>
+      </c>
       <c r="U94" s="2" t="s">
         <v>27</v>
       </c>
@@ -13832,49 +13854,49 @@
         <v>280</v>
       </c>
       <c r="F219" s="5">
-        <v>0.56999999999999995</v>
+        <v>0.59</v>
       </c>
       <c r="G219" s="5">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="H219" s="5">
-        <v>0.57999999999999996</v>
+        <v>0.59</v>
       </c>
       <c r="I219" s="5">
-        <v>0.61</v>
+        <v>0.63</v>
       </c>
       <c r="J219" s="5">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="K219" s="5">
         <v>0.69</v>
       </c>
       <c r="L219" s="5">
-        <v>0.67</v>
+        <v>0.69</v>
       </c>
       <c r="M219" s="5">
         <v>0.69</v>
       </c>
       <c r="N219" s="5">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="O219" s="5">
+        <v>0.78</v>
+      </c>
+      <c r="P219" s="5">
+        <v>0.77</v>
+      </c>
+      <c r="Q219" s="5">
         <v>0.81</v>
       </c>
-      <c r="P219" s="5">
-        <v>0.81</v>
-      </c>
-      <c r="Q219" s="5">
-        <v>0.86</v>
-      </c>
       <c r="R219" s="5">
-        <v>0.98</v>
+        <v>0.85</v>
       </c>
       <c r="S219" s="5">
-        <v>1.18</v>
+        <v>0.9</v>
       </c>
       <c r="T219" s="5">
-        <v>1.38</v>
+        <v>0.97</v>
       </c>
       <c r="U219" s="2" t="s">
         <v>271</v>
@@ -23259,49 +23281,49 @@
         <v>280</v>
       </c>
       <c r="F376" s="5">
-        <v>0.56999999999999995</v>
+        <v>0.59</v>
       </c>
       <c r="G376" s="5">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="H376" s="5">
-        <v>0.57999999999999996</v>
+        <v>0.59</v>
       </c>
       <c r="I376" s="5">
-        <v>0.61</v>
+        <v>0.63</v>
       </c>
       <c r="J376" s="5">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="K376" s="5">
         <v>0.69</v>
       </c>
       <c r="L376" s="5">
-        <v>0.67</v>
+        <v>0.69</v>
       </c>
       <c r="M376" s="5">
         <v>0.69</v>
       </c>
       <c r="N376" s="5">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="O376" s="5">
+        <v>0.78</v>
+      </c>
+      <c r="P376" s="5">
+        <v>0.77</v>
+      </c>
+      <c r="Q376" s="5">
         <v>0.81</v>
       </c>
-      <c r="P376" s="5">
-        <v>0.81</v>
-      </c>
-      <c r="Q376" s="5">
-        <v>0.86</v>
-      </c>
       <c r="R376" s="5">
-        <v>0.98</v>
+        <v>0.85</v>
       </c>
       <c r="S376" s="5">
-        <v>1.18</v>
+        <v>0.9</v>
       </c>
       <c r="T376" s="5">
-        <v>1.38</v>
+        <v>0.97</v>
       </c>
       <c r="U376" s="2" t="s">
         <v>271</v>
@@ -29102,7 +29124,7 @@
     <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.39370078740157499" right="0.39370078740157499" top="0.39370078740157499" bottom="0.39370078740157499" header="0.39370078740157499" footer="0.39370078740157499"/>
-  <pageSetup paperSize="9" scale="70" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="71" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Okno serwisowe 10.03 - poprawa
</commit_message>
<xml_diff>
--- a/assets/excel/en/global_sdg_indicators.xlsx
+++ b/assets/excel/en/global_sdg_indicators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dregerj\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD0C22C0-2E09-4E0C-AB67-95CFA5FF22C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C45C18D-27C3-4B0A-9794-E86C23747C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -871,7 +871,7 @@
     <t>8.4.1 Resource productivity - PROXY!</t>
   </si>
   <si>
-    <t>euro per kilogram [euro/kg]</t>
+    <t>Euro per kilogram, chain linked volumes (2015)</t>
   </si>
   <si>
     <t>8.4.2 Domestic material consumption (DMC)</t>
@@ -1729,7 +1729,7 @@
     <t>100% deaths registration</t>
   </si>
   <si>
-    <t>Last update: 10-03-2026, 12:34</t>
+    <t>Last update: 17-03-2026, 07:49</t>
   </si>
 </sst>
 </file>
@@ -13837,7 +13837,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="219" spans="1:21" ht="27" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>275</v>
       </c>
@@ -23264,7 +23264,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="376" spans="1:21" ht="27" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A376" s="2" t="s">
         <v>428</v>
       </c>

</xml_diff>

<commit_message>
Okno serwisowe - aktualizacja Excel
</commit_message>
<xml_diff>
--- a/assets/excel/en/global_sdg_indicators.xlsx
+++ b/assets/excel/en/global_sdg_indicators.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dregerj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sidwab\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C45C18D-27C3-4B0A-9794-E86C23747C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9851D111-D78D-4B73-A273-EFC436C835CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -658,7 +658,7 @@
     <t>5.2.1 Percentage of women aged 18-74 who have experienced physical, sexual or psychological violence from a current or former partner - PROXY!</t>
   </si>
   <si>
-    <t>European Union Agency for Fundamental Rights</t>
+    <t>Eurostat, European Union Agency for Fundamental Rights</t>
   </si>
   <si>
     <t>5.3.1 Number of concluded marriages in which the woman on her wedding day was below 18 years - PROXY!</t>
@@ -877,6 +877,9 @@
     <t>8.4.2 Domestic material consumption (DMC)</t>
   </si>
   <si>
+    <t>total in thousands</t>
+  </si>
+  <si>
     <t>tonnes</t>
   </si>
   <si>
@@ -1324,9 +1327,6 @@
     <t>12.2.2 Domestic Material Consumption (DMC)</t>
   </si>
   <si>
-    <t>thous. tonnes, tonnes</t>
-  </si>
-  <si>
     <t>12.4.1 Number of parties to international multilateral environmental agreements on hazardous waste, and other chemicals that meet their commitments and obligations in transmitting information as required by each relevant agreement</t>
   </si>
   <si>
@@ -1729,7 +1729,7 @@
     <t>100% deaths registration</t>
   </si>
   <si>
-    <t>Last update: 17-03-2026, 07:49</t>
+    <t>Last update: 24-03-2026, 11:46</t>
   </si>
 </sst>
 </file>
@@ -10735,9 +10735,7 @@
       </c>
       <c r="F155" s="3"/>
       <c r="G155" s="3"/>
-      <c r="H155" s="6">
-        <v>2</v>
-      </c>
+      <c r="H155" s="3"/>
       <c r="I155" s="3"/>
       <c r="J155" s="3"/>
       <c r="K155" s="3"/>
@@ -10746,7 +10744,9 @@
       <c r="N155" s="3"/>
       <c r="O155" s="3"/>
       <c r="P155" s="3"/>
-      <c r="Q155" s="3"/>
+      <c r="Q155" s="4">
+        <v>14.6</v>
+      </c>
       <c r="R155" s="3"/>
       <c r="S155" s="3"/>
       <c r="T155" s="3"/>
@@ -11771,7 +11771,9 @@
         <v>46.1</v>
       </c>
       <c r="S177" s="3"/>
-      <c r="T177" s="3"/>
+      <c r="T177" s="4">
+        <v>50.2</v>
+      </c>
       <c r="U177" s="2" t="s">
         <v>27</v>
       </c>
@@ -11820,7 +11822,9 @@
         <v>33.1</v>
       </c>
       <c r="S178" s="3"/>
-      <c r="T178" s="3"/>
+      <c r="T178" s="4">
+        <v>33.700000000000003</v>
+      </c>
       <c r="U178" s="2" t="s">
         <v>27</v>
       </c>
@@ -11869,7 +11873,9 @@
         <v>42.4</v>
       </c>
       <c r="S179" s="3"/>
-      <c r="T179" s="3"/>
+      <c r="T179" s="4">
+        <v>44.1</v>
+      </c>
       <c r="U179" s="2" t="s">
         <v>27</v>
       </c>
@@ -11918,7 +11924,9 @@
         <v>32.299999999999997</v>
       </c>
       <c r="S180" s="3"/>
-      <c r="T180" s="3"/>
+      <c r="T180" s="4">
+        <v>32.9</v>
+      </c>
       <c r="U180" s="2" t="s">
         <v>27</v>
       </c>
@@ -11967,7 +11975,9 @@
         <v>56.3</v>
       </c>
       <c r="S181" s="3"/>
-      <c r="T181" s="3"/>
+      <c r="T181" s="4">
+        <v>57</v>
+      </c>
       <c r="U181" s="2" t="s">
         <v>27</v>
       </c>
@@ -12016,7 +12026,9 @@
         <v>35.4</v>
       </c>
       <c r="S182" s="3"/>
-      <c r="T182" s="3"/>
+      <c r="T182" s="4">
+        <v>36.6</v>
+      </c>
       <c r="U182" s="2" t="s">
         <v>27</v>
       </c>
@@ -12065,7 +12077,9 @@
         <v>59.7</v>
       </c>
       <c r="S183" s="3"/>
-      <c r="T183" s="3"/>
+      <c r="T183" s="4">
+        <v>59.6</v>
+      </c>
       <c r="U183" s="2" t="s">
         <v>27</v>
       </c>
@@ -13913,10 +13927,10 @@
         <v>24</v>
       </c>
       <c r="D220" s="3" t="s">
-        <v>25</v>
+        <v>282</v>
       </c>
       <c r="E220" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F220" s="4">
         <v>627714.30000000005</v>
@@ -13978,10 +13992,10 @@
         <v>24</v>
       </c>
       <c r="D221" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E221" s="3" t="s">
         <v>283</v>
-      </c>
-      <c r="E221" s="3" t="s">
-        <v>282</v>
       </c>
       <c r="F221" s="5">
         <v>16.5</v>
@@ -14037,7 +14051,7 @@
         <v>275</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C222" s="2" t="s">
         <v>32</v>
@@ -14046,7 +14060,7 @@
         <v>25</v>
       </c>
       <c r="E222" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F222" s="5">
         <v>21.98</v>
@@ -14086,7 +14100,7 @@
         <v>275</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C223" s="2" t="s">
         <v>32</v>
@@ -14095,7 +14109,7 @@
         <v>33</v>
       </c>
       <c r="E223" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F223" s="5">
         <v>22.89</v>
@@ -14135,7 +14149,7 @@
         <v>275</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C224" s="2" t="s">
         <v>32</v>
@@ -14144,7 +14158,7 @@
         <v>34</v>
       </c>
       <c r="E224" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F224" s="5">
         <v>21</v>
@@ -14184,16 +14198,16 @@
         <v>275</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D225" s="3" t="s">
         <v>231</v>
       </c>
       <c r="E225" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F225" s="5">
         <v>43.51</v>
@@ -14233,16 +14247,16 @@
         <v>275</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C226" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D226" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E226" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D226" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="E226" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="F226" s="5">
         <v>31.84</v>
@@ -14282,16 +14296,16 @@
         <v>275</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C227" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D227" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E227" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D227" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="E227" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="F227" s="5">
         <v>21.77</v>
@@ -14331,16 +14345,16 @@
         <v>275</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C228" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D228" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="E228" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D228" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="E228" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="F228" s="5">
         <v>17.649999999999999</v>
@@ -14380,16 +14394,16 @@
         <v>275</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C229" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D229" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="E229" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D229" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="E229" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="F229" s="5">
         <v>12.44</v>
@@ -14429,16 +14443,16 @@
         <v>275</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C230" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D230" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="E230" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D230" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="E230" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="F230" s="5">
         <v>12.82</v>
@@ -14478,16 +14492,16 @@
         <v>275</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C231" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D231" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="E231" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D231" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="E231" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="F231" s="5">
         <v>16.059999999999999</v>
@@ -14527,16 +14541,16 @@
         <v>275</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C232" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D232" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="E232" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D232" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E232" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="F232" s="5">
         <v>17.239999999999998</v>
@@ -14576,16 +14590,16 @@
         <v>275</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C233" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D233" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="E233" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D233" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="E233" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="F233" s="5">
         <v>12.22</v>
@@ -14625,16 +14639,16 @@
         <v>275</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D234" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E234" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F234" s="5">
         <v>13.71</v>
@@ -14674,16 +14688,16 @@
         <v>275</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D235" s="3" t="s">
         <v>182</v>
       </c>
       <c r="E235" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F235" s="5">
         <v>20.66</v>
@@ -14723,16 +14737,16 @@
         <v>275</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D236" s="3" t="s">
         <v>183</v>
       </c>
       <c r="E236" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F236" s="5">
         <v>24.33</v>
@@ -14772,16 +14786,16 @@
         <v>275</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D237" s="3" t="s">
         <v>184</v>
       </c>
       <c r="E237" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F237" s="5">
         <v>22.3</v>
@@ -14821,16 +14835,16 @@
         <v>275</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D238" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E238" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F238" s="5">
         <v>22.61</v>
@@ -14870,16 +14884,16 @@
         <v>275</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D239" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E239" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F239" s="5">
         <v>27.21</v>
@@ -14919,16 +14933,16 @@
         <v>275</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D240" s="3" t="s">
         <v>41</v>
       </c>
       <c r="E240" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F240" s="5">
         <v>32.57</v>
@@ -14968,7 +14982,7 @@
         <v>275</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C241" s="2" t="s">
         <v>32</v>
@@ -15033,7 +15047,7 @@
         <v>275</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C242" s="2" t="s">
         <v>32</v>
@@ -15098,7 +15112,7 @@
         <v>275</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C243" s="2" t="s">
         <v>32</v>
@@ -15163,13 +15177,13 @@
         <v>275</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C244" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D244" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E244" s="3" t="s">
         <v>26</v>
@@ -15228,7 +15242,7 @@
         <v>275</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C245" s="2" t="s">
         <v>35</v>
@@ -15293,7 +15307,7 @@
         <v>275</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>35</v>
@@ -15358,7 +15372,7 @@
         <v>275</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C247" s="2" t="s">
         <v>35</v>
@@ -15423,13 +15437,13 @@
         <v>275</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C248" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D248" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E248" s="3" t="s">
         <v>26</v>
@@ -15488,10 +15502,10 @@
         <v>275</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D249" s="3" t="s">
         <v>25</v>
@@ -15553,7 +15567,7 @@
         <v>275</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C250" s="2" t="s">
         <v>24</v>
@@ -15618,7 +15632,7 @@
         <v>275</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C251" s="2" t="s">
         <v>48</v>
@@ -15681,13 +15695,13 @@
         <v>275</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C252" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D252" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E252" s="3" t="s">
         <v>49</v>
@@ -15744,13 +15758,13 @@
         <v>275</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D253" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E253" s="3" t="s">
         <v>150</v>
@@ -15779,7 +15793,7 @@
       <c r="S253" s="3"/>
       <c r="T253" s="3"/>
       <c r="U253" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="254" spans="1:21" ht="36" x14ac:dyDescent="0.25">
@@ -15787,13 +15801,13 @@
         <v>275</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D254" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E254" s="3" t="s">
         <v>150</v>
@@ -15822,7 +15836,7 @@
       <c r="S254" s="3"/>
       <c r="T254" s="3"/>
       <c r="U254" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="255" spans="1:21" ht="36" x14ac:dyDescent="0.25">
@@ -15830,13 +15844,13 @@
         <v>275</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D255" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E255" s="3" t="s">
         <v>150</v>
@@ -15865,7 +15879,7 @@
       <c r="S255" s="3"/>
       <c r="T255" s="3"/>
       <c r="U255" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="256" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -15873,7 +15887,7 @@
         <v>275</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C256" s="2" t="s">
         <v>24</v>
@@ -15938,7 +15952,7 @@
         <v>275</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C257" s="2" t="s">
         <v>24</v>
@@ -15947,7 +15961,7 @@
         <v>25</v>
       </c>
       <c r="E257" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F257" s="4">
         <v>85.8</v>
@@ -15989,7 +16003,7 @@
       <c r="S257" s="3"/>
       <c r="T257" s="3"/>
       <c r="U257" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="258" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -15997,7 +16011,7 @@
         <v>275</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C258" s="2" t="s">
         <v>32</v>
@@ -16026,7 +16040,7 @@
       <c r="S258" s="3"/>
       <c r="T258" s="3"/>
       <c r="U258" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="259" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -16034,7 +16048,7 @@
         <v>275</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C259" s="2" t="s">
         <v>32</v>
@@ -16063,7 +16077,7 @@
       <c r="S259" s="3"/>
       <c r="T259" s="3"/>
       <c r="U259" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="260" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -16071,7 +16085,7 @@
         <v>275</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C260" s="2" t="s">
         <v>32</v>
@@ -16100,7 +16114,7 @@
       <c r="S260" s="3"/>
       <c r="T260" s="3"/>
       <c r="U260" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="261" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -16108,13 +16122,13 @@
         <v>275</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C261" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D261" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E261" s="3" t="s">
         <v>26</v>
@@ -16137,7 +16151,7 @@
       <c r="S261" s="3"/>
       <c r="T261" s="3"/>
       <c r="U261" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="262" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -16145,7 +16159,7 @@
         <v>275</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C262" s="2" t="s">
         <v>35</v>
@@ -16174,7 +16188,7 @@
       <c r="S262" s="3"/>
       <c r="T262" s="3"/>
       <c r="U262" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="263" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -16182,7 +16196,7 @@
         <v>275</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C263" s="2" t="s">
         <v>35</v>
@@ -16211,7 +16225,7 @@
       <c r="S263" s="3"/>
       <c r="T263" s="3"/>
       <c r="U263" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="264" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -16219,7 +16233,7 @@
         <v>275</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C264" s="2" t="s">
         <v>35</v>
@@ -16248,7 +16262,7 @@
       <c r="S264" s="3"/>
       <c r="T264" s="3"/>
       <c r="U264" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="265" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -16256,13 +16270,13 @@
         <v>275</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C265" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D265" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E265" s="3" t="s">
         <v>26</v>
@@ -16285,7 +16299,7 @@
       <c r="S265" s="3"/>
       <c r="T265" s="3"/>
       <c r="U265" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="266" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -16293,7 +16307,7 @@
         <v>275</v>
       </c>
       <c r="B266" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C266" s="2" t="s">
         <v>24</v>
@@ -16343,19 +16357,19 @@
     </row>
     <row r="267" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B267" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D267" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E267" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F267" s="6">
         <v>261314</v>
@@ -16408,19 +16422,19 @@
     </row>
     <row r="268" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A268" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B268" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D268" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="E268" s="3" t="s">
         <v>325</v>
-      </c>
-      <c r="E268" s="3" t="s">
-        <v>324</v>
       </c>
       <c r="F268" s="6">
         <v>569652</v>
@@ -16473,19 +16487,19 @@
     </row>
     <row r="269" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D269" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E269" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F269" s="6">
         <v>671</v>
@@ -16538,19 +16552,19 @@
     </row>
     <row r="270" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A270" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D270" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E270" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F270" s="6">
         <v>1397</v>
@@ -16603,19 +16617,19 @@
     </row>
     <row r="271" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A271" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B271" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D271" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E271" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F271" s="6">
         <v>4990</v>
@@ -16668,19 +16682,19 @@
     </row>
     <row r="272" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B272" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D272" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E272" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F272" s="6">
         <v>234568</v>
@@ -16733,19 +16747,19 @@
     </row>
     <row r="273" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A273" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D273" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="E273" s="3" t="s">
         <v>325</v>
-      </c>
-      <c r="E273" s="3" t="s">
-        <v>324</v>
       </c>
       <c r="F273" s="6">
         <v>1491253</v>
@@ -16798,19 +16812,19 @@
     </row>
     <row r="274" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A274" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B274" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D274" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E274" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F274" s="6">
         <v>56208</v>
@@ -16863,19 +16877,19 @@
     </row>
     <row r="275" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A275" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B275" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D275" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E275" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F275" s="6">
         <v>8362</v>
@@ -16928,19 +16942,19 @@
     </row>
     <row r="276" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A276" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D276" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E276" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F276" s="6">
         <v>5141</v>
@@ -16993,19 +17007,19 @@
     </row>
     <row r="277" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A277" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B277" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C277" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="D277" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="D277" s="3" t="s">
-        <v>328</v>
-      </c>
       <c r="E277" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F277" s="6">
         <v>41</v>
@@ -17058,10 +17072,10 @@
     </row>
     <row r="278" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A278" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C278" s="2" t="s">
         <v>24</v>
@@ -17123,10 +17137,10 @@
     </row>
     <row r="279" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C279" s="2" t="s">
         <v>24</v>
@@ -17186,10 +17200,10 @@
     </row>
     <row r="280" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B280" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C280" s="2" t="s">
         <v>24</v>
@@ -17249,13 +17263,13 @@
     </row>
     <row r="281" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A281" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D281" s="3" t="s">
         <v>25</v>
@@ -17307,21 +17321,21 @@
       </c>
       <c r="T281" s="3"/>
       <c r="U281" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="282" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A282" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D282" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E282" s="3" t="s">
         <v>26</v>
@@ -17370,21 +17384,21 @@
       </c>
       <c r="T282" s="3"/>
       <c r="U282" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="283" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A283" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B283" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D283" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E283" s="3" t="s">
         <v>26</v>
@@ -17433,18 +17447,18 @@
       </c>
       <c r="T283" s="3"/>
       <c r="U283" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="284" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A284" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B284" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D284" s="3" t="s">
         <v>25</v>
@@ -17496,21 +17510,21 @@
       </c>
       <c r="T284" s="3"/>
       <c r="U284" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="285" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A285" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B285" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D285" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E285" s="3" t="s">
         <v>26</v>
@@ -17559,21 +17573,21 @@
       </c>
       <c r="T285" s="3"/>
       <c r="U285" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="286" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A286" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C286" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="D286" s="3" t="s">
         <v>339</v>
-      </c>
-      <c r="D286" s="3" t="s">
-        <v>338</v>
       </c>
       <c r="E286" s="3" t="s">
         <v>26</v>
@@ -17622,15 +17636,15 @@
       </c>
       <c r="T286" s="3"/>
       <c r="U286" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="287" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A287" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B287" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C287" s="2" t="s">
         <v>24</v>
@@ -17639,7 +17653,7 @@
         <v>25</v>
       </c>
       <c r="E287" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F287" s="5">
         <v>0.38</v>
@@ -17675,15 +17689,15 @@
       <c r="S287" s="3"/>
       <c r="T287" s="3"/>
       <c r="U287" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="288" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A288" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C288" s="2" t="s">
         <v>24</v>
@@ -17743,10 +17757,10 @@
     </row>
     <row r="289" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A289" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B289" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C289" s="2" t="s">
         <v>24</v>
@@ -17755,7 +17769,7 @@
         <v>25</v>
       </c>
       <c r="E289" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F289" s="4">
         <v>1674.9</v>
@@ -17806,10 +17820,10 @@
     </row>
     <row r="290" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C290" s="2" t="s">
         <v>24</v>
@@ -17865,10 +17879,10 @@
     </row>
     <row r="291" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A291" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B291" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C291" s="2" t="s">
         <v>24</v>
@@ -17920,16 +17934,16 @@
     </row>
     <row r="292" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A292" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D292" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E292" s="3" t="s">
         <v>26</v>
@@ -17973,16 +17987,16 @@
     </row>
     <row r="293" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A293" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D293" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E293" s="3" t="s">
         <v>26</v>
@@ -18028,13 +18042,13 @@
     </row>
     <row r="294" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A294" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B294" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D294" s="3" t="s">
         <v>25</v>
@@ -18093,16 +18107,16 @@
     </row>
     <row r="295" spans="1:21" ht="63" x14ac:dyDescent="0.25">
       <c r="A295" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B295" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D295" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E295" s="3" t="s">
         <v>26</v>
@@ -18158,10 +18172,10 @@
     </row>
     <row r="296" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A296" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B296" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C296" s="2" t="s">
         <v>32</v>
@@ -18223,10 +18237,10 @@
     </row>
     <row r="297" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A297" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C297" s="2" t="s">
         <v>32</v>
@@ -18288,10 +18302,10 @@
     </row>
     <row r="298" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A298" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B298" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C298" s="2" t="s">
         <v>32</v>
@@ -18353,16 +18367,16 @@
     </row>
     <row r="299" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A299" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B299" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C299" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D299" s="3" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E299" s="3" t="s">
         <v>26</v>
@@ -18418,16 +18432,16 @@
     </row>
     <row r="300" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A300" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B300" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C300" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D300" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E300" s="3" t="s">
         <v>26</v>
@@ -18483,10 +18497,10 @@
     </row>
     <row r="301" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A301" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C301" s="2" t="s">
         <v>35</v>
@@ -18548,10 +18562,10 @@
     </row>
     <row r="302" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A302" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C302" s="2" t="s">
         <v>35</v>
@@ -18613,10 +18627,10 @@
     </row>
     <row r="303" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A303" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B303" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C303" s="2" t="s">
         <v>35</v>
@@ -18678,10 +18692,10 @@
     </row>
     <row r="304" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A304" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C304" s="2" t="s">
         <v>35</v>
@@ -18743,10 +18757,10 @@
     </row>
     <row r="305" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A305" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C305" s="2" t="s">
         <v>24</v>
@@ -18784,10 +18798,10 @@
     </row>
     <row r="306" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A306" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C306" s="2" t="s">
         <v>24</v>
@@ -18847,16 +18861,16 @@
     </row>
     <row r="307" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A307" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D307" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E307" s="3" t="s">
         <v>26</v>
@@ -18907,21 +18921,21 @@
         <v>20.3</v>
       </c>
       <c r="U307" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="308" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A308" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D308" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E308" s="3" t="s">
         <v>26</v>
@@ -18972,21 +18986,21 @@
         <v>-1</v>
       </c>
       <c r="U308" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="309" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A309" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B309" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D309" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E309" s="3" t="s">
         <v>26</v>
@@ -19037,21 +19051,21 @@
         <v>18.899999999999999</v>
       </c>
       <c r="U309" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="310" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A310" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B310" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D310" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E310" s="3" t="s">
         <v>26</v>
@@ -19102,21 +19116,21 @@
         <v>4.2</v>
       </c>
       <c r="U310" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="311" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A311" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B311" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D311" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E311" s="3" t="s">
         <v>26</v>
@@ -19167,21 +19181,21 @@
         <v>1.8</v>
       </c>
       <c r="U311" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="312" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A312" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B312" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D312" s="3" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E312" s="3" t="s">
         <v>26</v>
@@ -19232,21 +19246,21 @@
         <v>57.2</v>
       </c>
       <c r="U312" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="313" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A313" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B313" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D313" s="3" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E313" s="3" t="s">
         <v>26</v>
@@ -19297,21 +19311,21 @@
         <v>1.7</v>
       </c>
       <c r="U313" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="314" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A314" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B314" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C314" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D314" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E314" s="3" t="s">
         <v>26</v>
@@ -19362,21 +19376,21 @@
         <v>14.7</v>
       </c>
       <c r="U314" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="315" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A315" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B315" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C315" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D315" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E315" s="3" t="s">
         <v>26</v>
@@ -19427,21 +19441,21 @@
         <v>72.099999999999994</v>
       </c>
       <c r="U315" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="316" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A316" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B316" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C316" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D316" s="3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E316" s="3" t="s">
         <v>26</v>
@@ -19492,21 +19506,21 @@
         <v>49.8</v>
       </c>
       <c r="U316" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="317" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A317" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B317" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C317" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D317" s="3" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E317" s="3" t="s">
         <v>26</v>
@@ -19557,21 +19571,21 @@
         <v>28</v>
       </c>
       <c r="U317" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="318" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A318" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B318" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C318" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D318" s="3" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E318" s="3" t="s">
         <v>26</v>
@@ -19622,15 +19636,15 @@
         <v>48</v>
       </c>
       <c r="U318" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="319" spans="1:21" ht="18" x14ac:dyDescent="0.25">
       <c r="A319" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B319" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C319" s="2" t="s">
         <v>24</v>
@@ -19687,21 +19701,21 @@
         <v>4.04</v>
       </c>
       <c r="U319" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="320" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A320" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C320" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D320" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E320" s="3" t="s">
         <v>95</v>
@@ -19752,21 +19766,21 @@
         <v>1840.15</v>
       </c>
       <c r="U320" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="321" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A321" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D321" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E321" s="3" t="s">
         <v>95</v>
@@ -19817,21 +19831,21 @@
         <v>705.25</v>
       </c>
       <c r="U321" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="322" spans="1:21" ht="54" x14ac:dyDescent="0.25">
       <c r="A322" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D322" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E322" s="3" t="s">
         <v>95</v>
@@ -19882,21 +19896,21 @@
         <v>12.96</v>
       </c>
       <c r="U322" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="323" spans="1:21" ht="63" x14ac:dyDescent="0.25">
       <c r="A323" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B323" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C323" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D323" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E323" s="3" t="s">
         <v>95</v>
@@ -19947,21 +19961,21 @@
         <v>1.79</v>
       </c>
       <c r="U323" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="324" spans="1:21" ht="63" x14ac:dyDescent="0.25">
       <c r="A324" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B324" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C324" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D324" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E324" s="3" t="s">
         <v>95</v>
@@ -20012,21 +20026,21 @@
         <v>199.97</v>
       </c>
       <c r="U324" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="325" spans="1:21" ht="72" x14ac:dyDescent="0.25">
       <c r="A325" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B325" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C325" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D325" s="3" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E325" s="3" t="s">
         <v>95</v>
@@ -20077,21 +20091,21 @@
         <v>87.2</v>
       </c>
       <c r="U325" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="326" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A326" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B326" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C326" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D326" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E326" s="3" t="s">
         <v>95</v>
@@ -20142,21 +20156,21 @@
         <v>3699.5</v>
       </c>
       <c r="U326" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="327" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A327" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B327" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D327" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E327" s="3" t="s">
         <v>95</v>
@@ -20207,21 +20221,21 @@
         <v>3.2</v>
       </c>
       <c r="U327" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="328" spans="1:21" ht="54" x14ac:dyDescent="0.25">
       <c r="A328" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B328" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C328" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D328" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E328" s="3" t="s">
         <v>95</v>
@@ -20272,21 +20286,21 @@
         <v>0</v>
       </c>
       <c r="U328" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="329" spans="1:21" ht="54" x14ac:dyDescent="0.25">
       <c r="A329" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B329" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C329" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D329" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E329" s="3" t="s">
         <v>95</v>
@@ -20337,21 +20351,21 @@
         <v>338.9</v>
       </c>
       <c r="U329" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="330" spans="1:21" ht="63" x14ac:dyDescent="0.25">
       <c r="A330" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B330" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D330" s="3" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E330" s="3" t="s">
         <v>95</v>
@@ -20402,15 +20416,15 @@
         <v>405.8</v>
       </c>
       <c r="U330" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="331" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A331" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B331" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C331" s="2" t="s">
         <v>29</v>
@@ -20466,10 +20480,10 @@
     </row>
     <row r="332" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A332" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B332" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C332" s="2" t="s">
         <v>29</v>
@@ -20525,10 +20539,10 @@
     </row>
     <row r="333" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A333" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B333" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C333" s="2" t="s">
         <v>29</v>
@@ -20584,10 +20598,10 @@
     </row>
     <row r="334" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A334" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B334" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C334" s="2" t="s">
         <v>48</v>
@@ -20644,15 +20658,15 @@
         <v>2.73</v>
       </c>
       <c r="U334" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="335" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A335" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B335" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C335" s="2" t="s">
         <v>48</v>
@@ -20709,21 +20723,21 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="U335" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="336" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A336" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B336" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D336" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E336" s="3" t="s">
         <v>26</v>
@@ -20779,16 +20793,16 @@
     </row>
     <row r="337" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A337" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D337" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E337" s="3" t="s">
         <v>26</v>
@@ -20844,16 +20858,16 @@
     </row>
     <row r="338" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A338" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B338" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D338" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E338" s="3" t="s">
         <v>26</v>
@@ -20909,16 +20923,16 @@
     </row>
     <row r="339" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A339" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B339" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D339" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E339" s="3" t="s">
         <v>26</v>
@@ -20974,19 +20988,19 @@
     </row>
     <row r="340" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A340" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B340" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C340" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D340" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E340" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F340" s="4">
         <v>27.7</v>
@@ -21039,19 +21053,19 @@
     </row>
     <row r="341" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A341" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B341" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D341" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="E341" s="3" t="s">
         <v>407</v>
-      </c>
-      <c r="E341" s="3" t="s">
-        <v>406</v>
       </c>
       <c r="F341" s="4">
         <v>29.6</v>
@@ -21104,19 +21118,19 @@
     </row>
     <row r="342" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A342" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D342" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E342" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F342" s="4">
         <v>50.5</v>
@@ -21169,19 +21183,19 @@
     </row>
     <row r="343" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A343" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B343" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D343" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E343" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F343" s="4">
         <v>65.8</v>
@@ -21234,19 +21248,19 @@
     </row>
     <row r="344" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B344" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D344" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E344" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F344" s="4">
         <v>57.7</v>
@@ -21299,19 +21313,19 @@
     </row>
     <row r="345" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A345" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B345" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D345" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E345" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F345" s="4">
         <v>31.2</v>
@@ -21364,19 +21378,19 @@
     </row>
     <row r="346" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B346" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D346" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E346" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F346" s="4">
         <v>25.4</v>
@@ -21429,19 +21443,19 @@
     </row>
     <row r="347" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A347" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B347" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D347" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E347" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F347" s="4">
         <v>38</v>
@@ -21494,19 +21508,19 @@
     </row>
     <row r="348" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A348" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B348" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D348" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E348" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F348" s="4">
         <v>54.9</v>
@@ -21559,19 +21573,19 @@
     </row>
     <row r="349" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A349" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B349" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D349" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E349" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F349" s="4">
         <v>23.7</v>
@@ -21624,19 +21638,19 @@
     </row>
     <row r="350" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A350" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B350" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C350" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D350" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E350" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F350" s="4">
         <v>27.7</v>
@@ -21689,19 +21703,19 @@
     </row>
     <row r="351" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A351" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B351" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C351" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D351" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E351" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F351" s="4">
         <v>42.5</v>
@@ -21754,19 +21768,19 @@
     </row>
     <row r="352" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A352" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B352" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C352" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D352" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E352" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F352" s="4">
         <v>50.9</v>
@@ -21819,19 +21833,19 @@
     </row>
     <row r="353" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A353" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B353" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C353" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D353" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="E353" s="3" t="s">
         <v>407</v>
-      </c>
-      <c r="E353" s="3" t="s">
-        <v>406</v>
       </c>
       <c r="F353" s="4">
         <v>25.1</v>
@@ -21884,19 +21898,19 @@
     </row>
     <row r="354" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A354" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B354" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C354" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D354" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E354" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F354" s="4">
         <v>26.2</v>
@@ -21949,19 +21963,19 @@
     </row>
     <row r="355" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A355" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B355" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D355" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E355" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F355" s="3"/>
       <c r="G355" s="4">
@@ -22012,19 +22026,19 @@
     </row>
     <row r="356" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A356" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B356" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D356" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E356" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F356" s="4">
         <v>44.3</v>
@@ -22077,19 +22091,19 @@
     </row>
     <row r="357" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A357" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B357" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D357" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E357" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F357" s="4">
         <v>19.3</v>
@@ -22142,19 +22156,19 @@
     </row>
     <row r="358" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A358" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B358" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C358" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D358" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E358" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F358" s="4">
         <v>20.3</v>
@@ -22207,19 +22221,19 @@
     </row>
     <row r="359" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A359" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B359" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C359" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D359" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E359" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F359" s="4">
         <v>30.9</v>
@@ -22272,19 +22286,19 @@
     </row>
     <row r="360" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A360" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B360" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C360" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D360" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E360" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F360" s="4">
         <v>34.799999999999997</v>
@@ -22337,19 +22351,19 @@
     </row>
     <row r="361" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A361" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B361" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C361" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D361" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E361" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F361" s="3"/>
       <c r="G361" s="4">
@@ -22400,19 +22414,19 @@
     </row>
     <row r="362" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A362" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B362" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C362" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D362" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E362" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F362" s="3"/>
       <c r="G362" s="4">
@@ -22463,19 +22477,19 @@
     </row>
     <row r="363" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A363" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B363" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C363" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="D363" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="D363" s="3" t="s">
-        <v>417</v>
-      </c>
       <c r="E363" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F363" s="3"/>
       <c r="G363" s="4">
@@ -22526,13 +22540,13 @@
     </row>
     <row r="364" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A364" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B364" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C364" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D364" s="3" t="s">
         <v>25</v>
@@ -22586,21 +22600,21 @@
         <v>98.72</v>
       </c>
       <c r="U364" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="365" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A365" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B365" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C365" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D365" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E365" s="3" t="s">
         <v>26</v>
@@ -22651,21 +22665,21 @@
         <v>100</v>
       </c>
       <c r="U365" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="366" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A366" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B366" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C366" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D366" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="E366" s="3" t="s">
         <v>26</v>
@@ -22716,21 +22730,21 @@
         <v>96.13</v>
       </c>
       <c r="U366" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="367" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A367" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B367" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C367" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D367" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="E367" s="3" t="s">
         <v>26</v>
@@ -22781,18 +22795,18 @@
         <v>99.18</v>
       </c>
       <c r="U367" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="368" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A368" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B368" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C368" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D368" s="3" t="s">
         <v>25</v>
@@ -22846,21 +22860,21 @@
         <v>99.8</v>
       </c>
       <c r="U368" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="369" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A369" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B369" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C369" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D369" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E369" s="3" t="s">
         <v>26</v>
@@ -22911,21 +22925,21 @@
         <v>99.8</v>
       </c>
       <c r="U369" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="370" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A370" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B370" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C370" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D370" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="E370" s="3" t="s">
         <v>26</v>
@@ -22976,21 +22990,21 @@
         <v>99.8</v>
       </c>
       <c r="U370" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="371" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A371" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B371" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C371" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="D371" s="3" t="s">
         <v>425</v>
-      </c>
-      <c r="D371" s="3" t="s">
-        <v>424</v>
       </c>
       <c r="E371" s="3" t="s">
         <v>26</v>
@@ -23041,15 +23055,15 @@
         <v>99.6</v>
       </c>
       <c r="U371" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="372" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A372" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B372" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C372" s="2" t="s">
         <v>53</v>
@@ -23101,10 +23115,10 @@
     </row>
     <row r="373" spans="1:21" ht="63" x14ac:dyDescent="0.25">
       <c r="A373" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B373" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C373" s="2" t="s">
         <v>53</v>
@@ -23156,10 +23170,10 @@
     </row>
     <row r="374" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A374" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B374" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C374" s="2" t="s">
         <v>24</v>
@@ -23211,10 +23225,10 @@
     </row>
     <row r="375" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A375" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B375" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C375" s="2" t="s">
         <v>24</v>
@@ -23266,10 +23280,10 @@
     </row>
     <row r="376" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A376" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B376" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C376" s="2" t="s">
         <v>24</v>
@@ -23331,19 +23345,19 @@
     </row>
     <row r="377" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A377" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C377" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D377" s="3" t="s">
-        <v>25</v>
+        <v>282</v>
       </c>
       <c r="E377" s="3" t="s">
-        <v>431</v>
+        <v>283</v>
       </c>
       <c r="F377" s="4">
         <v>627714.30000000005</v>
@@ -23396,19 +23410,19 @@
     </row>
     <row r="378" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A378" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B378" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C378" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D378" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E378" s="3" t="s">
         <v>283</v>
-      </c>
-      <c r="E378" s="3" t="s">
-        <v>431</v>
       </c>
       <c r="F378" s="5">
         <v>16.5</v>
@@ -23461,7 +23475,7 @@
     </row>
     <row r="379" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A379" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B379" s="2" t="s">
         <v>432</v>
@@ -23526,7 +23540,7 @@
     </row>
     <row r="380" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A380" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B380" s="2" t="s">
         <v>434</v>
@@ -23575,7 +23589,7 @@
     </row>
     <row r="381" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A381" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B381" s="2" t="s">
         <v>434</v>
@@ -23622,7 +23636,7 @@
     </row>
     <row r="382" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A382" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B382" s="2" t="s">
         <v>434</v>
@@ -23669,7 +23683,7 @@
     </row>
     <row r="383" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A383" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B383" s="2" t="s">
         <v>440</v>
@@ -23728,7 +23742,7 @@
     </row>
     <row r="384" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A384" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B384" s="2" t="s">
         <v>443</v>
@@ -23779,7 +23793,7 @@
     </row>
     <row r="385" spans="1:21" ht="27" x14ac:dyDescent="0.25">
       <c r="A385" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B385" s="2" t="s">
         <v>445</v>
@@ -23844,7 +23858,7 @@
     </row>
     <row r="386" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A386" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B386" s="2" t="s">
         <v>447</v>
@@ -27849,7 +27863,7 @@
         <v>1</v>
       </c>
       <c r="U457" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="458" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -28321,7 +28335,7 @@
         <v>548</v>
       </c>
       <c r="E465" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F465" s="6">
         <v>37896</v>
@@ -28386,7 +28400,7 @@
         <v>549</v>
       </c>
       <c r="E466" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F466" s="4">
         <v>103.2</v>
@@ -28451,7 +28465,7 @@
         <v>550</v>
       </c>
       <c r="E467" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F467" s="4">
         <v>102.6</v>
@@ -28516,7 +28530,7 @@
         <v>551</v>
       </c>
       <c r="E468" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F468" s="4">
         <v>19.600000000000001</v>
@@ -28581,7 +28595,7 @@
         <v>552</v>
       </c>
       <c r="E469" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F469" s="4">
         <v>53.7</v>
@@ -28646,7 +28660,7 @@
         <v>553</v>
       </c>
       <c r="E470" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F470" s="4">
         <v>-7.4</v>
@@ -29124,7 +29138,7 @@
     <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.39370078740157499" right="0.39370078740157499" top="0.39370078740157499" bottom="0.39370078740157499" header="0.39370078740157499" footer="0.39370078740157499"/>
-  <pageSetup paperSize="9" scale="71" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="70" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Okno serwisowe - aktualizacja plików Excel i PDF
</commit_message>
<xml_diff>
--- a/assets/excel/en/global_sdg_indicators.xlsx
+++ b/assets/excel/en/global_sdg_indicators.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sidwab\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7952798-5690-4B12-A06B-1EB0E455A291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F05A8087-F568-4366-BB49-09FA8E1C3995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SDGs_1-17" sheetId="1" r:id="rId1"/>
@@ -1723,7 +1723,7 @@
     <t>100% deaths registration</t>
   </si>
   <si>
-    <t>Last update: 23-06-2026, 13:15</t>
+    <t>Last update: 07-07-2026, 14:01</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Okno serwisowe - pliki excel
</commit_message>
<xml_diff>
--- a/assets/excel/en/global_sdg_indicators.xlsx
+++ b/assets/excel/en/global_sdg_indicators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\niewiadomskaew\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E02A16B5-9439-4008-9911-9EEF5ACB9CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C7705C0-2613-472D-86E0-9929EDFB9EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2857" uniqueCount="566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2857" uniqueCount="564">
   <si>
     <t>sdg.gov.pl/en</t>
   </si>
@@ -1531,15 +1531,9 @@
     <t>number of crimes</t>
   </si>
   <si>
-    <t>women</t>
-  </si>
-  <si>
     <t>ascertained crimes against persons aged 0-14 - by sex</t>
   </si>
   <si>
-    <t>men</t>
-  </si>
-  <si>
     <t>ascertained crimes against persons aged 0-17 - by legal qualification</t>
   </si>
   <si>
@@ -1726,7 +1720,7 @@
     <t>100% deaths registration</t>
   </si>
   <si>
-    <t>Last update: 26-08-2026, 12:35</t>
+    <t>Last update: 01-09-2026, 14:01</t>
   </si>
 </sst>
 </file>
@@ -1828,7 +1822,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
@@ -1852,6 +1846,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2296,14 +2293,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10"/>
-      <c r="B1" s="10"/>
+      <c r="A1" s="11"/>
+      <c r="B1" s="11"/>
     </row>
     <row r="2" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="10"/>
+      <c r="B2" s="11"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -8931,7 +8928,7 @@
         <v>34</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>157</v>
+        <v>35</v>
       </c>
       <c r="E110" s="3" t="s">
         <v>28</v>
@@ -8974,7 +8971,7 @@
         <v>34</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>158</v>
+        <v>36</v>
       </c>
       <c r="E111" s="3" t="s">
         <v>28</v>
@@ -10549,7 +10546,9 @@
       <c r="U143" s="6">
         <v>1</v>
       </c>
-      <c r="V143" s="3"/>
+      <c r="V143" s="9">
+        <v>1</v>
+      </c>
       <c r="W143" s="2" t="s">
         <v>192</v>
       </c>
@@ -24964,7 +24963,9 @@
       <c r="U384" s="6">
         <v>1</v>
       </c>
-      <c r="V384" s="3"/>
+      <c r="V384" s="9">
+        <v>1</v>
+      </c>
       <c r="W384" s="2" t="s">
         <v>192</v>
       </c>
@@ -25541,7 +25542,9 @@
       <c r="U393" s="6">
         <v>1</v>
       </c>
-      <c r="V393" s="3"/>
+      <c r="V393" s="9">
+        <v>1</v>
+      </c>
       <c r="W393" s="2" t="s">
         <v>192</v>
       </c>
@@ -27241,7 +27244,7 @@
         <v>498</v>
       </c>
       <c r="D422" s="3" t="s">
-        <v>500</v>
+        <v>36</v>
       </c>
       <c r="E422" s="3" t="s">
         <v>499</v>
@@ -27295,7 +27298,7 @@
         <v>497</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D423" s="3" t="s">
         <v>27</v>
@@ -27352,10 +27355,10 @@
         <v>497</v>
       </c>
       <c r="C424" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D424" s="3" t="s">
-        <v>502</v>
+        <v>35</v>
       </c>
       <c r="E424" s="3" t="s">
         <v>499</v>
@@ -27409,10 +27412,10 @@
         <v>497</v>
       </c>
       <c r="C425" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D425" s="3" t="s">
-        <v>500</v>
+        <v>36</v>
       </c>
       <c r="E425" s="3" t="s">
         <v>499</v>
@@ -27466,10 +27469,10 @@
         <v>497</v>
       </c>
       <c r="C426" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="D426" s="3" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="E426" s="3" t="s">
         <v>499</v>
@@ -27523,10 +27526,10 @@
         <v>497</v>
       </c>
       <c r="C427" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="D427" s="3" t="s">
         <v>503</v>
-      </c>
-      <c r="D427" s="3" t="s">
-        <v>505</v>
       </c>
       <c r="E427" s="3" t="s">
         <v>499</v>
@@ -27580,10 +27583,10 @@
         <v>497</v>
       </c>
       <c r="C428" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="D428" s="3" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="E428" s="3" t="s">
         <v>499</v>
@@ -27637,10 +27640,10 @@
         <v>497</v>
       </c>
       <c r="C429" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="D429" s="3" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="E429" s="3" t="s">
         <v>499</v>
@@ -27691,7 +27694,7 @@
         <v>490</v>
       </c>
       <c r="B430" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C430" s="2" t="s">
         <v>34</v>
@@ -27752,7 +27755,7 @@
       </c>
       <c r="V430" s="3"/>
       <c r="W430" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="431" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -27760,7 +27763,7 @@
         <v>490</v>
       </c>
       <c r="B431" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C431" s="2" t="s">
         <v>34</v>
@@ -27821,7 +27824,7 @@
       </c>
       <c r="V431" s="3"/>
       <c r="W431" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="432" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -27829,7 +27832,7 @@
         <v>490</v>
       </c>
       <c r="B432" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C432" s="2" t="s">
         <v>34</v>
@@ -27890,7 +27893,7 @@
       </c>
       <c r="V432" s="3"/>
       <c r="W432" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="433" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -27898,13 +27901,13 @@
         <v>490</v>
       </c>
       <c r="B433" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C433" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D433" s="3" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="E433" s="3" t="s">
         <v>28</v>
@@ -27959,7 +27962,7 @@
       </c>
       <c r="V433" s="3"/>
       <c r="W433" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="434" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -27967,13 +27970,13 @@
         <v>490</v>
       </c>
       <c r="B434" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C434" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D434" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="E434" s="3" t="s">
         <v>28</v>
@@ -28028,7 +28031,7 @@
       </c>
       <c r="V434" s="3"/>
       <c r="W434" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="435" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -28036,7 +28039,7 @@
         <v>490</v>
       </c>
       <c r="B435" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C435" s="2" t="s">
         <v>26</v>
@@ -28045,7 +28048,7 @@
         <v>27</v>
       </c>
       <c r="E435" s="3" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="F435" s="6">
         <v>12487</v>
@@ -28095,7 +28098,7 @@
       <c r="U435" s="3"/>
       <c r="V435" s="3"/>
       <c r="W435" s="2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="436" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28103,10 +28106,10 @@
         <v>490</v>
       </c>
       <c r="B436" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C436" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D436" s="3" t="s">
         <v>223</v>
@@ -28140,7 +28143,7 @@
       <c r="U436" s="3"/>
       <c r="V436" s="3"/>
       <c r="W436" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="437" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28148,10 +28151,10 @@
         <v>490</v>
       </c>
       <c r="B437" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C437" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D437" s="3" t="s">
         <v>225</v>
@@ -28185,7 +28188,7 @@
       <c r="U437" s="3"/>
       <c r="V437" s="3"/>
       <c r="W437" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="438" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28193,13 +28196,13 @@
         <v>490</v>
       </c>
       <c r="B438" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C438" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D438" s="3" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="E438" s="3" t="s">
         <v>28</v>
@@ -28230,7 +28233,7 @@
       <c r="U438" s="3"/>
       <c r="V438" s="3"/>
       <c r="W438" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="439" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28238,13 +28241,13 @@
         <v>490</v>
       </c>
       <c r="B439" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C439" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="D439" s="3" t="s">
         <v>518</v>
-      </c>
-      <c r="D439" s="3" t="s">
-        <v>520</v>
       </c>
       <c r="E439" s="3" t="s">
         <v>28</v>
@@ -28275,7 +28278,7 @@
       <c r="U439" s="3"/>
       <c r="V439" s="3"/>
       <c r="W439" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="440" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28283,13 +28286,13 @@
         <v>490</v>
       </c>
       <c r="B440" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C440" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D440" s="3" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="E440" s="3" t="s">
         <v>28</v>
@@ -28320,7 +28323,7 @@
       <c r="U440" s="3"/>
       <c r="V440" s="3"/>
       <c r="W440" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="441" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28328,13 +28331,13 @@
         <v>490</v>
       </c>
       <c r="B441" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C441" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D441" s="3" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="E441" s="3" t="s">
         <v>28</v>
@@ -28365,7 +28368,7 @@
       <c r="U441" s="3"/>
       <c r="V441" s="3"/>
       <c r="W441" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="442" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28373,10 +28376,10 @@
         <v>490</v>
       </c>
       <c r="B442" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C442" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D442" s="3" t="s">
         <v>42</v>
@@ -28410,7 +28413,7 @@
       <c r="U442" s="3"/>
       <c r="V442" s="3"/>
       <c r="W442" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="443" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28418,13 +28421,13 @@
         <v>490</v>
       </c>
       <c r="B443" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C443" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D443" s="3" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="E443" s="3" t="s">
         <v>28</v>
@@ -28455,7 +28458,7 @@
       <c r="U443" s="3"/>
       <c r="V443" s="3"/>
       <c r="W443" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="444" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28463,13 +28466,13 @@
         <v>490</v>
       </c>
       <c r="B444" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C444" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D444" s="3" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="E444" s="3" t="s">
         <v>28</v>
@@ -28500,7 +28503,7 @@
       <c r="U444" s="3"/>
       <c r="V444" s="3"/>
       <c r="W444" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="445" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28508,13 +28511,13 @@
         <v>490</v>
       </c>
       <c r="B445" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C445" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D445" s="3" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="E445" s="3" t="s">
         <v>28</v>
@@ -28545,7 +28548,7 @@
       <c r="U445" s="3"/>
       <c r="V445" s="3"/>
       <c r="W445" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="446" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28553,13 +28556,13 @@
         <v>490</v>
       </c>
       <c r="B446" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C446" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D446" s="3" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="E446" s="3" t="s">
         <v>28</v>
@@ -28590,7 +28593,7 @@
       <c r="U446" s="3"/>
       <c r="V446" s="3"/>
       <c r="W446" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="447" spans="1:23" ht="36" x14ac:dyDescent="0.25">
@@ -28598,10 +28601,10 @@
         <v>490</v>
       </c>
       <c r="B447" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C447" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D447" s="3" t="s">
         <v>42</v>
@@ -28635,7 +28638,7 @@
       <c r="U447" s="3"/>
       <c r="V447" s="3"/>
       <c r="W447" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="448" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -28643,7 +28646,7 @@
         <v>490</v>
       </c>
       <c r="B448" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C448" s="2" t="s">
         <v>26</v>
@@ -28704,7 +28707,7 @@
       </c>
       <c r="V448" s="3"/>
       <c r="W448" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="449" spans="1:23" ht="27" x14ac:dyDescent="0.25">
@@ -28712,7 +28715,7 @@
         <v>490</v>
       </c>
       <c r="B449" s="2" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C449" s="2" t="s">
         <v>26</v>
@@ -28752,10 +28755,10 @@
     </row>
     <row r="450" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A450" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B450" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C450" s="2" t="s">
         <v>26</v>
@@ -28821,10 +28824,10 @@
     </row>
     <row r="451" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A451" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B451" s="2" t="s">
         <v>527</v>
-      </c>
-      <c r="B451" s="2" t="s">
-        <v>529</v>
       </c>
       <c r="C451" s="2" t="s">
         <v>26</v>
@@ -28890,13 +28893,13 @@
     </row>
     <row r="452" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A452" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B452" s="2" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C452" s="2" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D452" s="3" t="s">
         <v>27</v>
@@ -28959,66 +28962,66 @@
     </row>
     <row r="453" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A453" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B453" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="C453" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="D453" s="3" t="s">
         <v>530</v>
-      </c>
-      <c r="C453" s="2" t="s">
-        <v>531</v>
-      </c>
-      <c r="D453" s="3" t="s">
-        <v>532</v>
       </c>
       <c r="E453" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F453" s="9">
+      <c r="F453" s="10">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="G453" s="9">
+      <c r="G453" s="10">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="H453" s="9">
+      <c r="H453" s="10">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="I453" s="9">
+      <c r="I453" s="10">
         <v>9.1999999999999998E-3</v>
       </c>
-      <c r="J453" s="9">
+      <c r="J453" s="10">
         <v>7.7000000000000002E-3</v>
       </c>
-      <c r="K453" s="9">
+      <c r="K453" s="10">
         <v>9.5999999999999992E-3</v>
       </c>
-      <c r="L453" s="9">
+      <c r="L453" s="10">
         <v>1.5900000000000001E-2</v>
       </c>
-      <c r="M453" s="9">
+      <c r="M453" s="10">
         <v>2.8E-3</v>
       </c>
-      <c r="N453" s="9">
+      <c r="N453" s="10">
         <v>1.3299999999999999E-2</v>
       </c>
-      <c r="O453" s="9">
+      <c r="O453" s="10">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="P453" s="9">
+      <c r="P453" s="10">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="Q453" s="9">
+      <c r="Q453" s="10">
         <v>5.3E-3</v>
       </c>
-      <c r="R453" s="9">
+      <c r="R453" s="10">
         <v>2.2000000000000001E-3</v>
       </c>
-      <c r="S453" s="9">
+      <c r="S453" s="10">
         <v>1E-3</v>
       </c>
-      <c r="T453" s="9">
+      <c r="T453" s="10">
         <v>2.0000000000000001E-4</v>
       </c>
-      <c r="U453" s="9">
+      <c r="U453" s="10">
         <v>1.5699999999999999E-2</v>
       </c>
       <c r="V453" s="3"/>
@@ -29028,10 +29031,10 @@
     </row>
     <row r="454" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A454" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B454" s="2" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C454" s="2" t="s">
         <v>26</v>
@@ -29092,15 +29095,15 @@
       </c>
       <c r="V454" s="3"/>
       <c r="W454" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="455" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A455" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B455" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C455" s="2" t="s">
         <v>26</v>
@@ -29166,10 +29169,10 @@
     </row>
     <row r="456" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A456" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B456" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="C456" s="2" t="s">
         <v>26</v>
@@ -29230,21 +29233,21 @@
       </c>
       <c r="V456" s="3"/>
       <c r="W456" s="2" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="457" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A457" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B457" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="C457" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="D457" s="3" t="s">
         <v>538</v>
-      </c>
-      <c r="C457" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="D457" s="3" t="s">
-        <v>540</v>
       </c>
       <c r="E457" s="3" t="s">
         <v>51</v>
@@ -29302,16 +29305,16 @@
     </row>
     <row r="458" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A458" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B458" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C458" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="D458" s="3" t="s">
         <v>539</v>
-      </c>
-      <c r="D458" s="3" t="s">
-        <v>541</v>
       </c>
       <c r="E458" s="3" t="s">
         <v>51</v>
@@ -29369,16 +29372,16 @@
     </row>
     <row r="459" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A459" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B459" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C459" s="2" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="D459" s="3" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="E459" s="3" t="s">
         <v>51</v>
@@ -29436,10 +29439,10 @@
     </row>
     <row r="460" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A460" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B460" s="2" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C460" s="2" t="s">
         <v>26</v>
@@ -29503,10 +29506,10 @@
     </row>
     <row r="461" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A461" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B461" s="2" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="C461" s="2" t="s">
         <v>26</v>
@@ -29572,10 +29575,10 @@
     </row>
     <row r="462" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A462" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B462" s="2" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C462" s="2" t="s">
         <v>26</v>
@@ -29641,16 +29644,16 @@
     </row>
     <row r="463" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A463" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B463" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C463" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D463" s="3" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="E463" s="3" t="s">
         <v>288</v>
@@ -29710,16 +29713,16 @@
     </row>
     <row r="464" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A464" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B464" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C464" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D464" s="3" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="E464" s="3" t="s">
         <v>288</v>
@@ -29779,16 +29782,16 @@
     </row>
     <row r="465" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A465" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B465" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C465" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D465" s="3" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="E465" s="3" t="s">
         <v>288</v>
@@ -29848,16 +29851,16 @@
     </row>
     <row r="466" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A466" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B466" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C466" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D466" s="3" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="E466" s="3" t="s">
         <v>288</v>
@@ -29917,16 +29920,16 @@
     </row>
     <row r="467" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A467" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B467" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C467" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D467" s="3" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="E467" s="3" t="s">
         <v>288</v>
@@ -29986,16 +29989,16 @@
     </row>
     <row r="468" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A468" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B468" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C468" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D468" s="3" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="E468" s="3" t="s">
         <v>288</v>
@@ -30055,10 +30058,10 @@
     </row>
     <row r="469" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A469" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B469" s="2" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="C469" s="2" t="s">
         <v>26</v>
@@ -30110,10 +30113,10 @@
     </row>
     <row r="470" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A470" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B470" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="C470" s="2" t="s">
         <v>26</v>
@@ -30179,10 +30182,10 @@
     </row>
     <row r="471" spans="1:23" ht="27" x14ac:dyDescent="0.25">
       <c r="A471" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B471" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C471" s="2" t="s">
         <v>26</v>
@@ -30248,10 +30251,10 @@
     </row>
     <row r="472" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A472" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B472" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="C472" s="2" t="s">
         <v>26</v>
@@ -30260,7 +30263,7 @@
         <v>27</v>
       </c>
       <c r="E472" s="3" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="F472" s="3"/>
       <c r="G472" s="3"/>
@@ -30306,21 +30309,21 @@
       </c>
       <c r="V472" s="3"/>
       <c r="W472" s="2" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
     </row>
     <row r="473" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A473" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B473" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="C473" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="D473" s="3" t="s">
         <v>559</v>
-      </c>
-      <c r="C473" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="D473" s="3" t="s">
-        <v>561</v>
       </c>
       <c r="E473" s="3" t="s">
         <v>191</v>
@@ -30347,21 +30350,21 @@
       <c r="U473" s="3"/>
       <c r="V473" s="3"/>
       <c r="W473" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="474" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A474" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B474" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C474" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D474" s="3" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="E474" s="3" t="s">
         <v>191</v>
@@ -30416,21 +30419,21 @@
       </c>
       <c r="V474" s="3"/>
       <c r="W474" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="475" spans="1:23" ht="36" x14ac:dyDescent="0.25">
       <c r="A475" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B475" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C475" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D475" s="3" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="E475" s="3" t="s">
         <v>191</v>
@@ -30485,15 +30488,15 @@
       </c>
       <c r="V475" s="3"/>
       <c r="W475" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="476" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="477" spans="1:23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A477" s="12" t="s">
-        <v>565</v>
-      </c>
-      <c r="B477" s="10"/>
+      <c r="A477" s="13" t="s">
+        <v>563</v>
+      </c>
+      <c r="B477" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:B3" xr:uid="{00000000-0001-0000-0000-000000000000}"/>

</xml_diff>